<commit_message>
bind sva & stop clock hex0 added
</commit_message>
<xml_diff>
--- a/Team9_ProjectVerif_Team13_Module5/documentacion/PlanVerificacion_Team9_to_Team13.xlsx
+++ b/Team9_ProjectVerif_Team13_Module5/documentacion/PlanVerificacion_Team9_to_Team13.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vivado\Team9_ProjectVerif_Team13_Module5\dv_designverification\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vivado\Team9_ProjectVerif_Team13_Module5\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE5A133-BEB4-4643-9AF9-62F5EB269DE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558D0177-B93B-48A6-9D07-8AB44A78460E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Testcases_Checks" sheetId="3" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
   <si>
     <t>Date</t>
   </si>
@@ -117,18 +117,12 @@
     <t>Conteo en Unidades de Segundo</t>
   </si>
   <si>
-    <t>counter_assigned_to_in_value_when_start_triggers</t>
-  </si>
-  <si>
     <t>CHECK</t>
   </si>
   <si>
     <t>accumulator_assigned_to_one_when_start_triggers</t>
   </si>
   <si>
-    <t xml:space="preserve"> Desbordamiento de min_units a Incremento de min_tens</t>
-  </si>
-  <si>
     <t>busy_asserted_while_done_not_set</t>
   </si>
   <si>
@@ -210,15 +204,6 @@
     <t>hex1 se incremente de 0 a 5 cada 10 ciclos de hex0.</t>
   </si>
   <si>
-    <t>Desbordamiento de sec_tens a Incremento de min_units</t>
-  </si>
-  <si>
-    <t>Verificar que después de 60 segundos, hex2 incremente.</t>
-  </si>
-  <si>
-    <t>hex2 sube 1 cada 60 segundos (cuando hex1 pasa de 5 a 0).</t>
-  </si>
-  <si>
     <t>SEÑALES A VERIFICAR POR EQUIPO 9</t>
   </si>
   <si>
@@ -259,6 +244,9 @@
   </si>
   <si>
     <t>0011000</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Desbordamiento de min_units e Incremento de min_tens</t>
   </si>
 </sst>
 </file>
@@ -939,7 +927,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="2.7086217492014397E-2"/>
+          <c:y val="0.12371401354239077"/>
+          <c:w val="0.95004310762048183"/>
+          <c:h val="0.75053598002111166"/>
+        </c:manualLayout>
+      </c:layout>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -1514,16 +1512,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>26565</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>148590</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>502920</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>590265</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>65955</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>563880</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1848,7 +1846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.33203125" style="5" customWidth="1"/>
@@ -1876,13 +1874,13 @@
         <v>7</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F1" s="22" t="s">
         <v>9</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H1" s="22" t="s">
         <v>8</v>
@@ -1902,13 +1900,13 @@
         <v>13</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E2" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="23" t="s">
         <v>39</v>
-      </c>
-      <c r="F2" s="23" t="s">
-        <v>41</v>
       </c>
       <c r="G2" s="27" t="s">
         <v>16</v>
@@ -1934,19 +1932,19 @@
         <v>31</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G3" s="28" t="s">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="H3" s="28" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I3" s="29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="41.4" x14ac:dyDescent="0.3">
@@ -1963,27 +1961,27 @@
         <v>31</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G4" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="I4" s="28" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="39.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:13" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>13</v>
@@ -1991,72 +1989,76 @@
       <c r="D5" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>38</v>
+      <c r="E5" s="16" t="s">
+        <v>42</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>55</v>
+        <v>39</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>20</v>
       </c>
       <c r="H5" s="28" t="s">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="I5" s="28" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="26.4" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="G6" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="28" t="s">
-        <v>19</v>
-      </c>
       <c r="I6" s="28" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="52.8" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+    </row>
+    <row r="7" spans="1:13" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="27" t="s">
-        <v>45</v>
+      <c r="G7" s="28" t="s">
+        <v>23</v>
       </c>
       <c r="H7" s="28" t="s">
         <v>46</v>
@@ -2064,57 +2066,24 @@
       <c r="I7" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-    </row>
-    <row r="8" spans="1:13" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="28" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" s="28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E12" s="10"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E14" s="10"/>
+      <c r="E8" s="9"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E11" s="10"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="E13" s="10"/>
     </row>
   </sheetData>
   <autoFilter ref="B1:D1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
@@ -2272,7 +2241,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>B2:B1009</xm:sqref>
+          <xm:sqref>B2:B1008</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000001000000}">
           <x14:formula1>
@@ -2281,7 +2250,7 @@
           <x14:formula2>
             <xm:f>0</xm:f>
           </x14:formula2>
-          <xm:sqref>D2:D1009</xm:sqref>
+          <xm:sqref>D2:D1008</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2306,28 +2275,28 @@
   <sheetData>
     <row r="1" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B1" s="40" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C1" s="40"/>
       <c r="D1" s="40"/>
       <c r="E1" s="31"/>
       <c r="F1" s="32" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="2:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="34" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C2" s="34" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D2" s="34" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E2" s="35"/>
       <c r="F2" s="32" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -2357,7 +2326,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D5" s="38">
         <v>24</v>
@@ -2368,7 +2337,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D6" s="38">
         <v>30</v>
@@ -2379,7 +2348,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D7" s="38">
         <v>19</v>
@@ -2390,7 +2359,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D8" s="38">
         <v>12</v>
@@ -2401,7 +2370,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D9" s="38">
         <v>2</v>
@@ -2412,7 +2381,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D10" s="38">
         <v>78</v>
@@ -2423,7 +2392,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D11" s="38">
         <v>0</v>
@@ -2434,7 +2403,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D12" s="38">
         <v>18</v>
@@ -2456,13 +2425,13 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.88671875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="22.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2622,33 +2591,33 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>